<commit_message>
added capacity_id to ev volumes data
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/check_investments.xlsx
+++ b/reconcile/storage/output/check_investments.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1815"/>
+  <dimension ref="A1:K1848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64594,6 +64594,1267 @@
         <v>2025</v>
       </c>
     </row>
+    <row r="1816">
+      <c r="A1816" s="1" t="n">
+        <v>1814</v>
+      </c>
+      <c r="B1816" t="inlineStr"/>
+      <c r="C1816" t="inlineStr"/>
+      <c r="D1816" t="inlineStr"/>
+      <c r="E1816" t="inlineStr"/>
+      <c r="F1816" t="inlineStr"/>
+      <c r="G1816" t="inlineStr"/>
+      <c r="H1816" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="I1816" t="inlineStr"/>
+      <c r="J1816" t="inlineStr"/>
+      <c r="K1816" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="1" t="n">
+        <v>1815</v>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>$111.02m (€103m)</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>02m</t>
+        </is>
+      </c>
+      <c r="D1817" t="inlineStr"/>
+      <c r="E1817" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F1817" t="n">
+        <v>111</v>
+      </c>
+      <c r="G1817" t="n">
+        <v>111</v>
+      </c>
+      <c r="H1817" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="I1817" t="n">
+        <v>102.6447198076568</v>
+      </c>
+      <c r="J1817" t="n">
+        <v>111</v>
+      </c>
+      <c r="K1817" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="1" t="n">
+        <v>1816</v>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>SEK10 billion (approximately $946 million)</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr"/>
+      <c r="D1818" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1818" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="F1818" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1818" t="n">
+        <v>10000000000</v>
+      </c>
+      <c r="H1818" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="I1818" t="n">
+        <v>882192070.8576671</v>
+      </c>
+      <c r="J1818" t="n">
+        <v>954002505.4254811</v>
+      </c>
+      <c r="K1818" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="1" t="n">
+        <v>1817</v>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>2.5m euros ($2.7m)</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="D1819" t="inlineStr"/>
+      <c r="E1819" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1819" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1819" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1819" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1819" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1819" t="n">
+        <v>2.1688</v>
+      </c>
+      <c r="K1819" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="1" t="n">
+        <v>1818</v>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>£423m</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr"/>
+      <c r="D1820" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1820" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1820" t="n">
+        <v>423</v>
+      </c>
+      <c r="G1820" t="n">
+        <v>423000000</v>
+      </c>
+      <c r="H1820" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1820" t="n">
+        <v>486514463.1663696</v>
+      </c>
+      <c r="J1820" t="n">
+        <v>512640289.8384036</v>
+      </c>
+      <c r="K1820" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="1" t="n">
+        <v>1819</v>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>£423m</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr"/>
+      <c r="D1821" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1821" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1821" t="n">
+        <v>423</v>
+      </c>
+      <c r="G1821" t="n">
+        <v>423000000</v>
+      </c>
+      <c r="H1821" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1821" t="n">
+        <v>486514463.1663696</v>
+      </c>
+      <c r="J1821" t="n">
+        <v>512640289.8384036</v>
+      </c>
+      <c r="K1821" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="1" t="n">
+        <v>1820</v>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>£423m</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr"/>
+      <c r="D1822" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1822" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1822" t="n">
+        <v>423</v>
+      </c>
+      <c r="G1822" t="n">
+        <v>423000000</v>
+      </c>
+      <c r="H1822" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1822" t="n">
+        <v>486514463.1663696</v>
+      </c>
+      <c r="J1822" t="n">
+        <v>512640289.8384036</v>
+      </c>
+      <c r="K1822" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="1" t="n">
+        <v>1821</v>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>up to £1.12bn</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>12bn</t>
+        </is>
+      </c>
+      <c r="D1823" t="inlineStr"/>
+      <c r="E1823" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1823" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="G1823" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="H1823" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1823" t="inlineStr">
+        <is>
+          <t>[None, 1.1501523951923631]</t>
+        </is>
+      </c>
+      <c r="J1823" t="inlineStr">
+        <is>
+          <t>[None, 1.211915578814193]</t>
+        </is>
+      </c>
+      <c r="K1823" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="1" t="n">
+        <v>1822</v>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>up to £1.12bn</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>12bn</t>
+        </is>
+      </c>
+      <c r="D1824" t="inlineStr"/>
+      <c r="E1824" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1824" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="G1824" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="H1824" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1824" t="inlineStr">
+        <is>
+          <t>[None, 1.1501523951923631]</t>
+        </is>
+      </c>
+      <c r="J1824" t="inlineStr">
+        <is>
+          <t>[None, 1.211915578814193]</t>
+        </is>
+      </c>
+      <c r="K1824" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="1" t="n">
+        <v>1823</v>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>up to £1.12bn</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>12bn</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr"/>
+      <c r="E1825" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1825" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="G1825" t="inlineStr">
+        <is>
+          <t>[None, 1.0]</t>
+        </is>
+      </c>
+      <c r="H1825" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1825" t="inlineStr">
+        <is>
+          <t>[None, 1.1501523951923631]</t>
+        </is>
+      </c>
+      <c r="J1825" t="inlineStr">
+        <is>
+          <t>[None, 1.211915578814193]</t>
+        </is>
+      </c>
+      <c r="K1825" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="1" t="n">
+        <v>1824</v>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>up to £3bn</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr"/>
+      <c r="D1826" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1826" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1826" t="inlineStr">
+        <is>
+          <t>[None, 3.0]</t>
+        </is>
+      </c>
+      <c r="G1826" t="inlineStr">
+        <is>
+          <t>[None, 3000000000.0]</t>
+        </is>
+      </c>
+      <c r="H1826" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1826" t="inlineStr">
+        <is>
+          <t>[None, 3450457185.5770893]</t>
+        </is>
+      </c>
+      <c r="J1826" t="inlineStr">
+        <is>
+          <t>[None, 3635746736.4425793]</t>
+        </is>
+      </c>
+      <c r="K1826" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="1" t="n">
+        <v>1825</v>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>up to £3bn</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr"/>
+      <c r="D1827" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1827" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1827" t="inlineStr">
+        <is>
+          <t>[None, 3.0]</t>
+        </is>
+      </c>
+      <c r="G1827" t="inlineStr">
+        <is>
+          <t>[None, 3000000000.0]</t>
+        </is>
+      </c>
+      <c r="H1827" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1827" t="inlineStr">
+        <is>
+          <t>[None, 3450457185.5770893]</t>
+        </is>
+      </c>
+      <c r="J1827" t="inlineStr">
+        <is>
+          <t>[None, 3635746736.4425793]</t>
+        </is>
+      </c>
+      <c r="K1827" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="1" t="n">
+        <v>1826</v>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>up to £3bn</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr"/>
+      <c r="D1828" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1828" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1828" t="inlineStr">
+        <is>
+          <t>[None, 3.0]</t>
+        </is>
+      </c>
+      <c r="G1828" t="inlineStr">
+        <is>
+          <t>[None, 3000000000.0]</t>
+        </is>
+      </c>
+      <c r="H1828" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1828" t="inlineStr">
+        <is>
+          <t>[None, 3450457185.5770893]</t>
+        </is>
+      </c>
+      <c r="J1828" t="inlineStr">
+        <is>
+          <t>[None, 3635746736.4425793]</t>
+        </is>
+      </c>
+      <c r="K1828" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="1" t="n">
+        <v>1827</v>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>EUR850m</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr"/>
+      <c r="D1829" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1829" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1829" t="n">
+        <v>850</v>
+      </c>
+      <c r="G1829" t="n">
+        <v>850000000</v>
+      </c>
+      <c r="H1829" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1829" t="n">
+        <v>850000000</v>
+      </c>
+      <c r="J1829" t="n">
+        <v>921740000</v>
+      </c>
+      <c r="K1829" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="1" t="n">
+        <v>1828</v>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>EUR600m</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr"/>
+      <c r="D1830" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1830" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1830" t="n">
+        <v>600</v>
+      </c>
+      <c r="G1830" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="H1830" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1830" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="J1830" t="n">
+        <v>650640000</v>
+      </c>
+      <c r="K1830" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="1" t="n">
+        <v>1829</v>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>EUR650m</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr"/>
+      <c r="D1831" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1831" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1831" t="n">
+        <v>650</v>
+      </c>
+      <c r="G1831" t="n">
+        <v>650000000</v>
+      </c>
+      <c r="H1831" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1831" t="n">
+        <v>650000000</v>
+      </c>
+      <c r="J1831" t="n">
+        <v>704860000</v>
+      </c>
+      <c r="K1831" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="1" t="n">
+        <v>1830</v>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>GBP250m</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr"/>
+      <c r="D1832" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1832" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1832" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1832" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="H1832" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="I1832" t="n">
+        <v>288779195.5766728</v>
+      </c>
+      <c r="J1832" t="n">
+        <v>304700555.2261333</v>
+      </c>
+      <c r="K1832" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="1" t="n">
+        <v>1831</v>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>GBP250m</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr"/>
+      <c r="D1833" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1833" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1833" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1833" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="H1833" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="I1833" t="n">
+        <v>288779195.5766728</v>
+      </c>
+      <c r="J1833" t="n">
+        <v>304700555.2261333</v>
+      </c>
+      <c r="K1833" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="1" t="n">
+        <v>1832</v>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>GBP250m</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr"/>
+      <c r="D1834" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1834" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1834" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1834" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="H1834" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="I1834" t="n">
+        <v>288779195.5766728</v>
+      </c>
+      <c r="J1834" t="n">
+        <v>304700555.2261333</v>
+      </c>
+      <c r="K1834" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="1" t="n">
+        <v>1833</v>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>EUR400m</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr"/>
+      <c r="D1835" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1835" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1835" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1835" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="H1835" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1835" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="J1835" t="n">
+        <v>421480000.0000001</v>
+      </c>
+      <c r="K1835" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="1" t="n">
+        <v>1834</v>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>£2.5 billion</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr"/>
+      <c r="D1836" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1836" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1836" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G1836" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="H1836" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="I1836" t="n">
+        <v>2887791955.766728</v>
+      </c>
+      <c r="J1836" t="n">
+        <v>3047005552.261333</v>
+      </c>
+      <c r="K1836" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="1" t="n">
+        <v>1835</v>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>GBP4bn</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr"/>
+      <c r="D1837" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1837" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1837" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1837" t="n">
+        <v>4000000000</v>
+      </c>
+      <c r="H1837" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1837" t="n">
+        <v>4600609580.769452</v>
+      </c>
+      <c r="J1837" t="n">
+        <v>4847662315.256772</v>
+      </c>
+      <c r="K1837" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="1" t="n">
+        <v>1836</v>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>GBP1bn</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr"/>
+      <c r="D1838" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1838" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1838" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1838" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="H1838" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1838" t="n">
+        <v>1150152395.192363</v>
+      </c>
+      <c r="J1838" t="n">
+        <v>1211915578.814193</v>
+      </c>
+      <c r="K1838" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="1" t="n">
+        <v>1837</v>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>GBP1bn</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr"/>
+      <c r="D1839" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1839" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1839" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1839" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="H1839" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1839" t="n">
+        <v>1150152395.192363</v>
+      </c>
+      <c r="J1839" t="n">
+        <v>1211915578.814193</v>
+      </c>
+      <c r="K1839" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="1" t="n">
+        <v>1838</v>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>EUR400m</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr"/>
+      <c r="D1840" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1840" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F1840" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1840" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="H1840" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1840" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="J1840" t="n">
+        <v>421480000.0000001</v>
+      </c>
+      <c r="K1840" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="1" t="n">
+        <v>1839</v>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>GBP3bn</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr"/>
+      <c r="D1841" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1841" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1841" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1841" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="H1841" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1841" t="n">
+        <v>3450457185.577089</v>
+      </c>
+      <c r="J1841" t="n">
+        <v>3635746736.442579</v>
+      </c>
+      <c r="K1841" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="1" t="n">
+        <v>1840</v>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>GBP3bn</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr"/>
+      <c r="D1842" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1842" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1842" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1842" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="H1842" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1842" t="n">
+        <v>3450457185.577089</v>
+      </c>
+      <c r="J1842" t="n">
+        <v>3635746736.442579</v>
+      </c>
+      <c r="K1842" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" s="1" t="n">
+        <v>1841</v>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>GBP3bn</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr"/>
+      <c r="D1843" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="E1843" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1843" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1843" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="H1843" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="I1843" t="n">
+        <v>3450457185.577089</v>
+      </c>
+      <c r="J1843" t="n">
+        <v>3635746736.442579</v>
+      </c>
+      <c r="K1843" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" s="1" t="n">
+        <v>1842</v>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>GBP100m</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr"/>
+      <c r="D1844" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1844" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1844" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1844" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H1844" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1844" t="n">
+        <v>116907105.6138792</v>
+      </c>
+      <c r="J1844" t="n">
+        <v>126774065.3276906</v>
+      </c>
+      <c r="K1844" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" s="1" t="n">
+        <v>1843</v>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>GBP100m</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr"/>
+      <c r="D1845" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1845" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1845" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1845" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H1845" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1845" t="n">
+        <v>116907105.6138792</v>
+      </c>
+      <c r="J1845" t="n">
+        <v>126774065.3276906</v>
+      </c>
+      <c r="K1845" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" s="1" t="n">
+        <v>1844</v>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>GBP100m</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr"/>
+      <c r="D1846" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1846" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1846" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1846" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H1846" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1846" t="n">
+        <v>116907105.6138792</v>
+      </c>
+      <c r="J1846" t="n">
+        <v>126774065.3276906</v>
+      </c>
+      <c r="K1846" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" s="1" t="n">
+        <v>1845</v>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>GBP100m</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr"/>
+      <c r="D1847" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1847" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1847" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1847" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H1847" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1847" t="n">
+        <v>116907105.6138792</v>
+      </c>
+      <c r="J1847" t="n">
+        <v>126774065.3276906</v>
+      </c>
+      <c r="K1847" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" s="1" t="n">
+        <v>1846</v>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>GBP100m</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr"/>
+      <c r="D1848" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E1848" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="F1848" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1848" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="H1848" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="I1848" t="n">
+        <v>116907105.6138792</v>
+      </c>
+      <c r="J1848" t="n">
+        <v>126774065.3276906</v>
+      </c>
+      <c r="K1848" t="n">
+        <v>2023</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
facility status updates if status different
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/check_investments.xlsx
+++ b/reconcile/storage/output/check_investments.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1991"/>
+  <dimension ref="A1:J2048"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64535,33 +64535,35 @@
     <row r="1956">
       <c r="A1956" t="inlineStr">
         <is>
-          <t>around two billion euros</t>
+          <t>50 million euro</t>
         </is>
       </c>
       <c r="B1956" t="inlineStr"/>
-      <c r="C1956" t="inlineStr"/>
+      <c r="C1956" t="n">
+        <v>1000000</v>
+      </c>
       <c r="D1956" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
       <c r="E1956" t="n">
-        <v>1000000000</v>
+        <v>50</v>
       </c>
       <c r="F1956" t="n">
-        <v>1000000000</v>
+        <v>50000000</v>
       </c>
       <c r="G1956" s="2" t="n">
-        <v>45352</v>
+        <v>45901</v>
       </c>
       <c r="H1956" t="n">
-        <v>1000000000</v>
+        <v>50000000</v>
       </c>
       <c r="I1956" t="n">
-        <v>1081300000</v>
+        <v>58270000</v>
       </c>
       <c r="J1956" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="1957">
@@ -64669,12 +64671,12 @@
     <row r="1960">
       <c r="A1960" t="inlineStr">
         <is>
-          <t>50 million euro</t>
+          <t>€1.8 billion</t>
         </is>
       </c>
       <c r="B1960" t="inlineStr"/>
       <c r="C1960" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D1960" t="inlineStr">
         <is>
@@ -64682,22 +64684,22 @@
         </is>
       </c>
       <c r="E1960" t="n">
-        <v>50</v>
+        <v>1.8</v>
       </c>
       <c r="F1960" t="n">
-        <v>50000000</v>
+        <v>1800000000</v>
       </c>
       <c r="G1960" s="2" t="n">
-        <v>45901</v>
+        <v>45597</v>
       </c>
       <c r="H1960" t="n">
-        <v>50000000</v>
+        <v>1800000000</v>
       </c>
       <c r="I1960" t="n">
-        <v>58270000</v>
+        <v>1959300000</v>
       </c>
       <c r="J1960" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1961">
@@ -64771,7 +64773,7 @@
     <row r="1963">
       <c r="A1963" t="inlineStr">
         <is>
-          <t>€1.8 billion</t>
+          <t>SEK 6.2 billion</t>
         </is>
       </c>
       <c r="B1963" t="inlineStr"/>
@@ -64780,60 +64782,60 @@
       </c>
       <c r="D1963" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SEK</t>
         </is>
       </c>
       <c r="E1963" t="n">
-        <v>1.8</v>
+        <v>6.2</v>
       </c>
       <c r="F1963" t="n">
-        <v>1800000000</v>
+        <v>6200000000</v>
       </c>
       <c r="G1963" s="2" t="n">
-        <v>45597</v>
+        <v>45231</v>
       </c>
       <c r="H1963" t="n">
-        <v>1800000000</v>
+        <v>525156699.9830595</v>
       </c>
       <c r="I1963" t="n">
-        <v>1959300000</v>
+        <v>553357614.7721499</v>
       </c>
       <c r="J1963" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
-          <t>SEK 6.2 billion</t>
+          <t>€13.6 million</t>
         </is>
       </c>
       <c r="B1964" t="inlineStr"/>
       <c r="C1964" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D1964" t="inlineStr">
         <is>
-          <t>SEK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="E1964" t="n">
-        <v>6.2</v>
+        <v>13.6</v>
       </c>
       <c r="F1964" t="n">
-        <v>6200000000</v>
+        <v>13600000</v>
       </c>
       <c r="G1964" s="2" t="n">
-        <v>45231</v>
+        <v>45901</v>
       </c>
       <c r="H1964" t="n">
-        <v>525156699.9830595</v>
+        <v>13600000</v>
       </c>
       <c r="I1964" t="n">
-        <v>553357614.7721499</v>
+        <v>15849440</v>
       </c>
       <c r="J1964" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="1965">
@@ -64907,12 +64909,12 @@
     <row r="1967">
       <c r="A1967" t="inlineStr">
         <is>
-          <t>€13.6 million</t>
+          <t>€1.65 billion</t>
         </is>
       </c>
       <c r="B1967" t="inlineStr"/>
       <c r="C1967" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D1967" t="inlineStr">
         <is>
@@ -64920,22 +64922,22 @@
         </is>
       </c>
       <c r="E1967" t="n">
-        <v>13.6</v>
+        <v>1.65</v>
       </c>
       <c r="F1967" t="n">
-        <v>13600000</v>
+        <v>1650000000</v>
       </c>
       <c r="G1967" s="2" t="n">
-        <v>45901</v>
+        <v>45474</v>
       </c>
       <c r="H1967" t="n">
-        <v>13600000</v>
+        <v>1650000000</v>
       </c>
       <c r="I1967" t="n">
-        <v>15849440</v>
+        <v>1772925000</v>
       </c>
       <c r="J1967" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1968">
@@ -65009,35 +65011,29 @@
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
-          <t>€1.65 billion</t>
-        </is>
-      </c>
-      <c r="B1970" t="inlineStr"/>
-      <c r="C1970" t="n">
-        <v>1000000000</v>
-      </c>
+          <t>single-digit billion-euro sum</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr">
+        <is>
+          <t>single digit billion</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr"/>
       <c r="D1970" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="E1970" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F1970" t="n">
-        <v>1650000000</v>
-      </c>
+      <c r="E1970" t="inlineStr"/>
+      <c r="F1970" t="inlineStr"/>
       <c r="G1970" s="2" t="n">
-        <v>45474</v>
-      </c>
-      <c r="H1970" t="n">
-        <v>1650000000</v>
-      </c>
-      <c r="I1970" t="n">
-        <v>1772925000</v>
-      </c>
+        <v>44713</v>
+      </c>
+      <c r="H1970" t="inlineStr"/>
+      <c r="I1970" t="inlineStr"/>
       <c r="J1970" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="1971">
@@ -65099,29 +65095,35 @@
     <row r="1973">
       <c r="A1973" t="inlineStr">
         <is>
-          <t>single-digit billion-euro sum</t>
-        </is>
-      </c>
-      <c r="B1973" t="inlineStr">
-        <is>
-          <t>single digit billion</t>
-        </is>
-      </c>
-      <c r="C1973" t="inlineStr"/>
+          <t>EUR 3.5 billion</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr"/>
+      <c r="C1973" t="n">
+        <v>1000000000</v>
+      </c>
       <c r="D1973" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="E1973" t="inlineStr"/>
-      <c r="F1973" t="inlineStr"/>
+      <c r="E1973" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F1973" t="n">
+        <v>3500000000</v>
+      </c>
       <c r="G1973" s="2" t="n">
-        <v>44713</v>
-      </c>
-      <c r="H1973" t="inlineStr"/>
-      <c r="I1973" t="inlineStr"/>
+        <v>45078</v>
+      </c>
+      <c r="H1973" t="n">
+        <v>3500000000</v>
+      </c>
+      <c r="I1973" t="n">
+        <v>3743950000</v>
+      </c>
       <c r="J1973" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="1974">
@@ -65229,7 +65231,7 @@
     <row r="1977">
       <c r="A1977" t="inlineStr">
         <is>
-          <t>EUR 3.5 billion</t>
+          <t>€1 billion</t>
         </is>
       </c>
       <c r="B1977" t="inlineStr"/>
@@ -65242,28 +65244,28 @@
         </is>
       </c>
       <c r="E1977" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="F1977" t="n">
-        <v>3500000000</v>
+        <v>1000000000</v>
       </c>
       <c r="G1977" s="2" t="n">
-        <v>45078</v>
+        <v>45352</v>
       </c>
       <c r="H1977" t="n">
-        <v>3500000000</v>
+        <v>1000000000</v>
       </c>
       <c r="I1977" t="n">
-        <v>3743950000</v>
+        <v>1081300000</v>
       </c>
       <c r="J1977" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1978">
       <c r="A1978" t="inlineStr">
         <is>
-          <t>€1 billion</t>
+          <t>€1.8 billion</t>
         </is>
       </c>
       <c r="B1978" t="inlineStr"/>
@@ -65276,19 +65278,19 @@
         </is>
       </c>
       <c r="E1978" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="F1978" t="n">
-        <v>1000000000</v>
+        <v>1800000000</v>
       </c>
       <c r="G1978" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="H1978" t="n">
-        <v>1000000000</v>
+        <v>1800000000</v>
       </c>
       <c r="I1978" t="n">
-        <v>1081300000</v>
+        <v>1946340000</v>
       </c>
       <c r="J1978" t="n">
         <v>2024</v>
@@ -65365,7 +65367,7 @@
     <row r="1981">
       <c r="A1981" t="inlineStr">
         <is>
-          <t>€1.8 billion</t>
+          <t>€1-1.5 billion</t>
         </is>
       </c>
       <c r="B1981" t="inlineStr"/>
@@ -65377,23 +65379,31 @@
           <t>EUR</t>
         </is>
       </c>
-      <c r="E1981" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F1981" t="n">
-        <v>1800000000</v>
+      <c r="E1981" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F1981" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
       </c>
       <c r="G1981" s="2" t="n">
-        <v>45352</v>
-      </c>
-      <c r="H1981" t="n">
-        <v>1800000000</v>
-      </c>
-      <c r="I1981" t="n">
-        <v>1946340000</v>
+        <v>44256</v>
+      </c>
+      <c r="H1981" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I1981" t="inlineStr">
+        <is>
+          <t>[1205300000.0, 1807950000.0]</t>
+        </is>
       </c>
       <c r="J1981" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="1982">
@@ -65693,43 +65703,33 @@
     <row r="1989">
       <c r="A1989" t="inlineStr">
         <is>
-          <t>€1-1.5 billion</t>
+          <t>two billion euros</t>
         </is>
       </c>
       <c r="B1989" t="inlineStr"/>
-      <c r="C1989" t="n">
-        <v>1000000000</v>
-      </c>
+      <c r="C1989" t="inlineStr"/>
       <c r="D1989" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="E1989" t="inlineStr">
-        <is>
-          <t>[1.0, 1.5]</t>
-        </is>
-      </c>
-      <c r="F1989" t="inlineStr">
-        <is>
-          <t>[1000000000.0, 1500000000.0]</t>
-        </is>
+      <c r="E1989" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F1989" t="n">
+        <v>1000000000</v>
       </c>
       <c r="G1989" s="2" t="n">
-        <v>44256</v>
-      </c>
-      <c r="H1989" t="inlineStr">
-        <is>
-          <t>[1000000000.0, 1500000000.0]</t>
-        </is>
-      </c>
-      <c r="I1989" t="inlineStr">
-        <is>
-          <t>[1205300000.0, 1807950000.0]</t>
-        </is>
+        <v>45231</v>
+      </c>
+      <c r="H1989" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I1989" t="n">
+        <v>1053700000</v>
       </c>
       <c r="J1989" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="1990">
@@ -65767,32 +65767,1910 @@
     <row r="1991">
       <c r="A1991" t="inlineStr">
         <is>
+          <t>EUR 165m</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr"/>
+      <c r="C1991" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D1991" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1991" t="n">
+        <v>165</v>
+      </c>
+      <c r="F1991" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="G1991" s="2" t="n">
+        <v>44317</v>
+      </c>
+      <c r="H1991" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="I1991" t="n">
+        <v>199144000</v>
+      </c>
+      <c r="J1991" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr">
+        <is>
+          <t>EUR 165m</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr"/>
+      <c r="C1992" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D1992" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1992" t="n">
+        <v>165</v>
+      </c>
+      <c r="F1992" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="G1992" s="2" t="n">
+        <v>44317</v>
+      </c>
+      <c r="H1992" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="I1992" t="n">
+        <v>199144000</v>
+      </c>
+      <c r="J1992" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr"/>
+      <c r="B1993" t="inlineStr"/>
+      <c r="C1993" t="inlineStr"/>
+      <c r="D1993" t="inlineStr"/>
+      <c r="E1993" t="inlineStr"/>
+      <c r="F1993" t="inlineStr"/>
+      <c r="G1993" s="2" t="n">
+        <v>44652</v>
+      </c>
+      <c r="H1993" t="inlineStr"/>
+      <c r="I1993" t="inlineStr"/>
+      <c r="J1993" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr"/>
+      <c r="B1994" t="inlineStr"/>
+      <c r="C1994" t="inlineStr"/>
+      <c r="D1994" t="inlineStr"/>
+      <c r="E1994" t="inlineStr"/>
+      <c r="F1994" t="inlineStr"/>
+      <c r="G1994" s="2" t="n">
+        <v>44652</v>
+      </c>
+      <c r="H1994" t="inlineStr"/>
+      <c r="I1994" t="inlineStr"/>
+      <c r="J1994" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>€55 million</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr"/>
+      <c r="C1995" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D1995" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1995" t="n">
+        <v>55</v>
+      </c>
+      <c r="F1995" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="G1995" s="2" t="n">
+        <v>45901</v>
+      </c>
+      <c r="H1995" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="I1995" t="n">
+        <v>64097000</v>
+      </c>
+      <c r="J1995" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>20 million euros</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr"/>
+      <c r="C1996" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D1996" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1996" t="n">
+        <v>20</v>
+      </c>
+      <c r="F1996" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="G1996" s="2" t="n">
+        <v>45017</v>
+      </c>
+      <c r="H1996" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="I1996" t="n">
+        <v>21746666.66666666</v>
+      </c>
+      <c r="J1996" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>$20.35m</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>35m</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr"/>
+      <c r="D1997" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E1997" t="n">
+        <v>20</v>
+      </c>
+      <c r="F1997" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1997" s="2" t="n">
+        <v>44743</v>
+      </c>
+      <c r="H1997" t="n">
+        <v>19.18465227817746</v>
+      </c>
+      <c r="I1997" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1997" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>€50 million</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr"/>
+      <c r="C1998" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D1998" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1998" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1998" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G1998" s="2" t="n">
+        <v>44378</v>
+      </c>
+      <c r="H1998" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="I1998" t="n">
+        <v>59419999.99999999</v>
+      </c>
+      <c r="J1998" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>€1 billion</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr"/>
+      <c r="C1999" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D1999" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E1999" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1999" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="G1999" s="2" t="n">
+        <v>44378</v>
+      </c>
+      <c r="H1999" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I1999" t="n">
+        <v>1188400000</v>
+      </c>
+      <c r="J1999" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>around two billion euros</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr"/>
+      <c r="C2000" t="inlineStr"/>
+      <c r="D2000" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2000" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F2000" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="G2000" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2000" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I2000" t="n">
+        <v>1081400000</v>
+      </c>
+      <c r="J2000" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>€2 billion</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr"/>
+      <c r="C2001" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2001" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2001" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2001" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="G2001" s="2" t="n">
+        <v>44805</v>
+      </c>
+      <c r="H2001" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="I2001" t="n">
+        <v>2000800000</v>
+      </c>
+      <c r="J2001" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>€2 billion</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr"/>
+      <c r="C2002" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2002" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2002" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2002" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="G2002" s="2" t="n">
+        <v>44805</v>
+      </c>
+      <c r="H2002" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="I2002" t="n">
+        <v>2000800000</v>
+      </c>
+      <c r="J2002" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
           <t>two billion euros</t>
         </is>
       </c>
-      <c r="B1991" t="inlineStr"/>
-      <c r="C1991" t="inlineStr"/>
-      <c r="D1991" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E1991" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="F1991" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="G1991" s="2" t="n">
-        <v>45231</v>
-      </c>
-      <c r="H1991" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="I1991" t="n">
-        <v>1053700000</v>
-      </c>
-      <c r="J1991" t="n">
+      <c r="B2003" t="inlineStr"/>
+      <c r="C2003" t="inlineStr"/>
+      <c r="D2003" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2003" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F2003" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="G2003" s="2" t="n">
+        <v>45261</v>
+      </c>
+      <c r="H2003" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I2003" t="n">
+        <v>1087500000</v>
+      </c>
+      <c r="J2003" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>two billion euros</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr"/>
+      <c r="C2004" t="inlineStr"/>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2004" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="F2004" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="G2004" s="2" t="n">
+        <v>45108</v>
+      </c>
+      <c r="H2004" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I2004" t="n">
+        <v>1087700000</v>
+      </c>
+      <c r="J2004" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>€74 million</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr"/>
+      <c r="C2005" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2005" t="n">
+        <v>74</v>
+      </c>
+      <c r="F2005" t="n">
+        <v>74000000</v>
+      </c>
+      <c r="G2005" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H2005" t="n">
+        <v>74000000</v>
+      </c>
+      <c r="I2005" t="n">
+        <v>79513000</v>
+      </c>
+      <c r="J2005" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>SEK 6.2 billion</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr"/>
+      <c r="C2006" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E2006" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F2006" t="n">
+        <v>6200000000</v>
+      </c>
+      <c r="G2006" s="2" t="n">
+        <v>45078</v>
+      </c>
+      <c r="H2006" t="n">
+        <v>532394487.1409557</v>
+      </c>
+      <c r="I2006" t="n">
+        <v>569502382.8946804</v>
+      </c>
+      <c r="J2006" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>SEK 400 million</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr"/>
+      <c r="C2007" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E2007" t="n">
+        <v>400</v>
+      </c>
+      <c r="F2007" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="G2007" s="2" t="n">
+        <v>45536</v>
+      </c>
+      <c r="H2007" t="n">
+        <v>35255233.19867793</v>
+      </c>
+      <c r="I2007" t="n">
+        <v>39026367.97649651</v>
+      </c>
+      <c r="J2007" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr"/>
+      <c r="B2008" t="inlineStr"/>
+      <c r="C2008" t="inlineStr"/>
+      <c r="D2008" t="inlineStr"/>
+      <c r="E2008" t="inlineStr"/>
+      <c r="F2008" t="inlineStr"/>
+      <c r="G2008" s="2" t="n">
+        <v>44927</v>
+      </c>
+      <c r="H2008" t="inlineStr"/>
+      <c r="I2008" t="inlineStr"/>
+      <c r="J2008" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>€4.2 billion</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr"/>
+      <c r="C2009" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2009" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F2009" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="G2009" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2009" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="I2009" t="n">
+        <v>4611390000</v>
+      </c>
+      <c r="J2009" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>€4.2 billion</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr"/>
+      <c r="C2010" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2010" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F2010" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="G2010" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2010" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="I2010" t="n">
+        <v>4611390000</v>
+      </c>
+      <c r="J2010" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>€4.2 billion</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr"/>
+      <c r="C2011" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2011" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F2011" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="G2011" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2011" t="n">
+        <v>4200000000</v>
+      </c>
+      <c r="I2011" t="n">
+        <v>4611390000</v>
+      </c>
+      <c r="J2011" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>€300 million</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr"/>
+      <c r="C2012" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2012" t="n">
+        <v>300</v>
+      </c>
+      <c r="F2012" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="G2012" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2012" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="I2012" t="n">
+        <v>329385000</v>
+      </c>
+      <c r="J2012" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>€300 million</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr"/>
+      <c r="C2013" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2013" t="n">
+        <v>300</v>
+      </c>
+      <c r="F2013" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="G2013" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2013" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="I2013" t="n">
+        <v>329385000</v>
+      </c>
+      <c r="J2013" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>€300 million</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr"/>
+      <c r="C2014" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2014" t="n">
+        <v>300</v>
+      </c>
+      <c r="F2014" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="G2014" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2014" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="I2014" t="n">
+        <v>329385000</v>
+      </c>
+      <c r="J2014" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>€250 million</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr"/>
+      <c r="C2015" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2015" t="n">
+        <v>250</v>
+      </c>
+      <c r="F2015" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="G2015" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2015" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="I2015" t="n">
+        <v>274487500</v>
+      </c>
+      <c r="J2015" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>€250 million</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr"/>
+      <c r="C2016" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2016" t="n">
+        <v>250</v>
+      </c>
+      <c r="F2016" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="G2016" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2016" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="I2016" t="n">
+        <v>274487500</v>
+      </c>
+      <c r="J2016" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>€250 million</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr"/>
+      <c r="C2017" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2017" t="n">
+        <v>250</v>
+      </c>
+      <c r="F2017" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="G2017" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2017" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="I2017" t="n">
+        <v>274487500</v>
+      </c>
+      <c r="J2017" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>€265m ($284m)</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr"/>
+      <c r="C2018" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2018" t="n">
+        <v>265</v>
+      </c>
+      <c r="F2018" t="n">
+        <v>265000000</v>
+      </c>
+      <c r="G2018" s="2" t="n">
+        <v>45444</v>
+      </c>
+      <c r="H2018" t="n">
+        <v>265000000</v>
+      </c>
+      <c r="I2018" t="n">
+        <v>287489666.6666667</v>
+      </c>
+      <c r="J2018" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>$150m</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr"/>
+      <c r="C2019" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E2019" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2019" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="G2019" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H2019" t="n">
+        <v>139387068.5970227</v>
+      </c>
+      <c r="I2019" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="J2019" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>$150m</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr"/>
+      <c r="C2020" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E2020" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2020" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="G2020" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H2020" t="n">
+        <v>139387068.5970227</v>
+      </c>
+      <c r="I2020" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="J2020" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr"/>
+      <c r="B2021" t="inlineStr"/>
+      <c r="C2021" t="inlineStr"/>
+      <c r="D2021" t="inlineStr"/>
+      <c r="E2021" t="inlineStr"/>
+      <c r="F2021" t="inlineStr"/>
+      <c r="G2021" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H2021" t="inlineStr"/>
+      <c r="I2021" t="inlineStr"/>
+      <c r="J2021" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr"/>
+      <c r="B2022" t="inlineStr"/>
+      <c r="C2022" t="inlineStr"/>
+      <c r="D2022" t="inlineStr"/>
+      <c r="E2022" t="inlineStr"/>
+      <c r="F2022" t="inlineStr"/>
+      <c r="G2022" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="H2022" t="inlineStr"/>
+      <c r="I2022" t="inlineStr"/>
+      <c r="J2022" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>€55 million</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr"/>
+      <c r="C2023" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2023" t="n">
+        <v>55</v>
+      </c>
+      <c r="F2023" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="G2023" s="2" t="n">
+        <v>44958</v>
+      </c>
+      <c r="H2023" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="I2023" t="n">
+        <v>59916999.99999999</v>
+      </c>
+      <c r="J2023" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>€1-1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr"/>
+      <c r="C2024" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2024" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F2024" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="G2024" s="2" t="n">
+        <v>44287</v>
+      </c>
+      <c r="H2024" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I2024" t="inlineStr">
+        <is>
+          <t>[1174600000.0, 1761900000.0000002]</t>
+        </is>
+      </c>
+      <c r="J2024" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>€1-1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr"/>
+      <c r="C2025" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2025" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F2025" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="G2025" s="2" t="n">
+        <v>44287</v>
+      </c>
+      <c r="H2025" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I2025" t="inlineStr">
+        <is>
+          <t>[1174600000.0, 1761900000.0000002]</t>
+        </is>
+      </c>
+      <c r="J2025" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>€1-1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr"/>
+      <c r="C2026" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2026" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F2026" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="G2026" s="2" t="n">
+        <v>44287</v>
+      </c>
+      <c r="H2026" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I2026" t="inlineStr">
+        <is>
+          <t>[1174600000.0, 1761900000.0000002]</t>
+        </is>
+      </c>
+      <c r="J2026" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>€1-1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr"/>
+      <c r="C2027" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2027" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F2027" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="G2027" s="2" t="n">
+        <v>44287</v>
+      </c>
+      <c r="H2027" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I2027" t="inlineStr">
+        <is>
+          <t>[1174600000.0, 1761900000.0000002]</t>
+        </is>
+      </c>
+      <c r="J2027" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>€2.5 billion</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr"/>
+      <c r="C2028" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2028" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2028" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="G2028" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="H2028" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="I2028" t="n">
+        <v>2742500000</v>
+      </c>
+      <c r="J2028" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>€2.5 billion</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr"/>
+      <c r="C2029" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2029" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2029" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="G2029" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="H2029" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="I2029" t="n">
+        <v>2742500000</v>
+      </c>
+      <c r="J2029" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>€2.5 billion</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr"/>
+      <c r="C2030" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2030" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2030" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="G2030" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="H2030" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="I2030" t="n">
+        <v>2742500000</v>
+      </c>
+      <c r="J2030" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>€2.5 billion</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr"/>
+      <c r="C2031" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2031" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2031" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="G2031" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="H2031" t="n">
+        <v>2500000000</v>
+      </c>
+      <c r="I2031" t="n">
+        <v>2742500000</v>
+      </c>
+      <c r="J2031" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr"/>
+      <c r="C2032" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2032" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2032" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2032" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2032" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2032" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2032" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr"/>
+      <c r="C2033" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2033" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2033" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2033" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2033" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2033" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2033" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr"/>
+      <c r="C2034" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2034" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2034" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2034" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2034" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2034" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2034" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr"/>
+      <c r="C2035" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2035" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2035" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2035" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2035" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2035" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2035" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr"/>
+      <c r="C2036" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2036" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2036" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2036" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2036" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2036" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2036" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr"/>
+      <c r="C2037" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2037" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2037" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2037" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2037" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2037" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2037" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr"/>
+      <c r="C2038" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2038" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2038" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2038" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2038" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2038" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2038" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>€1.3 billion</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr"/>
+      <c r="C2039" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2039" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F2039" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="G2039" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="H2039" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="I2039" t="n">
+        <v>1405820000</v>
+      </c>
+      <c r="J2039" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>EUR € 50 million</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr"/>
+      <c r="C2040" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2040" t="n">
+        <v>50</v>
+      </c>
+      <c r="F2040" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G2040" s="2" t="n">
+        <v>44256</v>
+      </c>
+      <c r="H2040" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="I2040" t="n">
+        <v>60265000</v>
+      </c>
+      <c r="J2040" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>EUR € 50 million</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr"/>
+      <c r="C2041" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2041" t="n">
+        <v>50</v>
+      </c>
+      <c r="F2041" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G2041" s="2" t="n">
+        <v>44256</v>
+      </c>
+      <c r="H2041" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="I2041" t="n">
+        <v>60265000</v>
+      </c>
+      <c r="J2041" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>€8 million ($8.7m)</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr"/>
+      <c r="C2042" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2042" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2042" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="G2042" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2042" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="I2042" t="n">
+        <v>8783600</v>
+      </c>
+      <c r="J2042" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>EUR 4.5 billion</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr"/>
+      <c r="C2043" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2043" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F2043" t="n">
+        <v>4500000000</v>
+      </c>
+      <c r="G2043" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="H2043" t="n">
+        <v>4500000000</v>
+      </c>
+      <c r="I2043" t="n">
+        <v>4842630000</v>
+      </c>
+      <c r="J2043" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>EUR 2.6 billion</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr"/>
+      <c r="C2044" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2044" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F2044" t="n">
+        <v>2600000000</v>
+      </c>
+      <c r="G2044" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2044" t="n">
+        <v>2600000000</v>
+      </c>
+      <c r="I2044" t="n">
+        <v>2854670000</v>
+      </c>
+      <c r="J2044" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>EUR 2.6 billion</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr"/>
+      <c r="C2045" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2045" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F2045" t="n">
+        <v>2600000000</v>
+      </c>
+      <c r="G2045" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="H2045" t="n">
+        <v>2600000000</v>
+      </c>
+      <c r="I2045" t="n">
+        <v>2854670000</v>
+      </c>
+      <c r="J2045" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>three million euros</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr"/>
+      <c r="C2046" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2046" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2046" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G2046" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="H2046" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="I2046" t="n">
+        <v>3291000</v>
+      </c>
+      <c r="J2046" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>EUR 1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr"/>
+      <c r="C2047" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2047" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F2047" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="G2047" s="2" t="n">
+        <v>44986</v>
+      </c>
+      <c r="H2047" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="I2047" t="n">
+        <v>1602600000</v>
+      </c>
+      <c r="J2047" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>EUR 1.5 billion</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr"/>
+      <c r="C2048" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2048" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F2048" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="G2048" s="2" t="n">
+        <v>44986</v>
+      </c>
+      <c r="H2048" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="I2048" t="n">
+        <v>1602600000</v>
+      </c>
+      <c r="J2048" t="n">
         <v>2023</v>
       </c>
     </row>

</xml_diff>

<commit_message>
calculate main from phase summaries direct
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/check_investments.xlsx
+++ b/reconcile/storage/output/check_investments.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2357"/>
+  <dimension ref="A1:J2356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76397,7 +76397,7 @@
     <row r="2319">
       <c r="A2319" t="inlineStr">
         <is>
-          <t>EUR 200 mn</t>
+          <t>€200 million</t>
         </is>
       </c>
       <c r="B2319" t="inlineStr"/>
@@ -76431,12 +76431,12 @@
     <row r="2320">
       <c r="A2320" t="inlineStr">
         <is>
-          <t>€200 million</t>
+          <t>€7 billion</t>
         </is>
       </c>
       <c r="B2320" t="inlineStr"/>
       <c r="C2320" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2320" t="inlineStr">
         <is>
@@ -76444,22 +76444,22 @@
         </is>
       </c>
       <c r="E2320" t="n">
-        <v>200</v>
+        <v>7</v>
       </c>
       <c r="F2320" t="n">
-        <v>200000000</v>
+        <v>7000000000</v>
       </c>
       <c r="G2320" s="2" t="n">
-        <v>45901</v>
+        <v>45444</v>
       </c>
       <c r="H2320" t="n">
-        <v>200000000</v>
+        <v>7000000000</v>
       </c>
       <c r="I2320" t="n">
-        <v>233080000</v>
+        <v>7594066666.666667</v>
       </c>
       <c r="J2320" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2321">
@@ -76567,12 +76567,12 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>€7 billion</t>
+          <t>EUR 1941 million</t>
         </is>
       </c>
       <c r="B2324" t="inlineStr"/>
       <c r="C2324" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2324" t="inlineStr">
         <is>
@@ -76580,62 +76580,62 @@
         </is>
       </c>
       <c r="E2324" t="n">
-        <v>7</v>
+        <v>1941</v>
       </c>
       <c r="F2324" t="n">
-        <v>7000000000</v>
+        <v>1941000000</v>
       </c>
       <c r="G2324" s="2" t="n">
-        <v>45444</v>
+        <v>44866</v>
       </c>
       <c r="H2324" t="n">
-        <v>7000000000</v>
+        <v>1941000000</v>
       </c>
       <c r="I2324" t="n">
-        <v>7594066666.666667</v>
+        <v>1930712700</v>
       </c>
       <c r="J2324" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>EUR 1941 million</t>
+          <t>1 billion pound ($1.33 billion)</t>
         </is>
       </c>
       <c r="B2325" t="inlineStr"/>
       <c r="C2325" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2325" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="E2325" t="n">
-        <v>1941</v>
+        <v>1</v>
       </c>
       <c r="F2325" t="n">
-        <v>1941000000</v>
+        <v>1000000000</v>
       </c>
       <c r="G2325" s="2" t="n">
-        <v>44866</v>
+        <v>45778</v>
       </c>
       <c r="H2325" t="n">
-        <v>1941000000</v>
+        <v>1172951733.036186</v>
       </c>
       <c r="I2325" t="n">
-        <v>1930712700</v>
+        <v>1332238578.3825</v>
       </c>
       <c r="J2325" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>1 billion pound ($1.33 billion)</t>
+          <t>£1bn</t>
         </is>
       </c>
       <c r="B2326" t="inlineStr"/>
@@ -76669,7 +76669,7 @@
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>£1bn</t>
+          <t>NOK 1.5 billion (USD 134m/EUR 128m)</t>
         </is>
       </c>
       <c r="B2327" t="inlineStr"/>
@@ -76678,60 +76678,60 @@
       </c>
       <c r="D2327" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="E2327" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F2327" t="n">
-        <v>1000000000</v>
+        <v>1500000000</v>
       </c>
       <c r="G2327" s="2" t="n">
-        <v>45778</v>
+        <v>45627</v>
       </c>
       <c r="H2327" t="n">
-        <v>1172951733.036186</v>
+        <v>128576939.0116719</v>
       </c>
       <c r="I2327" t="n">
-        <v>1332238578.3825</v>
+        <v>135331514.2077518</v>
       </c>
       <c r="J2327" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>NOK 1.5 billion (USD 134m/EUR 128m)</t>
+          <t>700 million euros</t>
         </is>
       </c>
       <c r="B2328" t="inlineStr"/>
       <c r="C2328" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2328" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="E2328" t="n">
-        <v>1.5</v>
+        <v>700</v>
       </c>
       <c r="F2328" t="n">
-        <v>1500000000</v>
+        <v>700000000</v>
       </c>
       <c r="G2328" s="2" t="n">
-        <v>45627</v>
+        <v>44713</v>
       </c>
       <c r="H2328" t="n">
-        <v>128576939.0116719</v>
+        <v>700000000</v>
       </c>
       <c r="I2328" t="n">
-        <v>135331514.2077518</v>
+        <v>749840000</v>
       </c>
       <c r="J2328" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2329">
@@ -76769,37 +76769,19 @@
       </c>
     </row>
     <row r="2330">
-      <c r="A2330" t="inlineStr">
-        <is>
-          <t>700 million euros</t>
-        </is>
-      </c>
+      <c r="A2330" t="inlineStr"/>
       <c r="B2330" t="inlineStr"/>
-      <c r="C2330" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D2330" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2330" t="n">
-        <v>700</v>
-      </c>
-      <c r="F2330" t="n">
-        <v>700000000</v>
-      </c>
+      <c r="C2330" t="inlineStr"/>
+      <c r="D2330" t="inlineStr"/>
+      <c r="E2330" t="inlineStr"/>
+      <c r="F2330" t="inlineStr"/>
       <c r="G2330" s="2" t="n">
-        <v>44713</v>
-      </c>
-      <c r="H2330" t="n">
-        <v>700000000</v>
-      </c>
-      <c r="I2330" t="n">
-        <v>749840000</v>
-      </c>
+        <v>45292</v>
+      </c>
+      <c r="H2330" t="inlineStr"/>
+      <c r="I2330" t="inlineStr"/>
       <c r="J2330" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2331">
@@ -76819,19 +76801,37 @@
       </c>
     </row>
     <row r="2332">
-      <c r="A2332" t="inlineStr"/>
+      <c r="A2332" t="inlineStr">
+        <is>
+          <t>EUR 1.5 billion</t>
+        </is>
+      </c>
       <c r="B2332" t="inlineStr"/>
-      <c r="C2332" t="inlineStr"/>
-      <c r="D2332" t="inlineStr"/>
-      <c r="E2332" t="inlineStr"/>
-      <c r="F2332" t="inlineStr"/>
+      <c r="C2332" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2332" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2332" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F2332" t="n">
+        <v>1500000000</v>
+      </c>
       <c r="G2332" s="2" t="n">
-        <v>45292</v>
-      </c>
-      <c r="H2332" t="inlineStr"/>
-      <c r="I2332" t="inlineStr"/>
+        <v>44986</v>
+      </c>
+      <c r="H2332" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="I2332" t="n">
+        <v>1602600000</v>
+      </c>
       <c r="J2332" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2333">
@@ -76871,7 +76871,7 @@
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>EUR 1.5 billion</t>
+          <t>€1 billion</t>
         </is>
       </c>
       <c r="B2334" t="inlineStr"/>
@@ -76884,19 +76884,19 @@
         </is>
       </c>
       <c r="E2334" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F2334" t="n">
-        <v>1500000000</v>
+        <v>1000000000</v>
       </c>
       <c r="G2334" s="2" t="n">
-        <v>44986</v>
+        <v>44958</v>
       </c>
       <c r="H2334" t="n">
-        <v>1500000000</v>
+        <v>1000000000</v>
       </c>
       <c r="I2334" t="n">
-        <v>1602600000</v>
+        <v>1089400000</v>
       </c>
       <c r="J2334" t="n">
         <v>2023</v>
@@ -76905,12 +76905,12 @@
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>€1 billion</t>
+          <t>600 million euros</t>
         </is>
       </c>
       <c r="B2335" t="inlineStr"/>
       <c r="C2335" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2335" t="inlineStr">
         <is>
@@ -76918,19 +76918,19 @@
         </is>
       </c>
       <c r="E2335" t="n">
-        <v>1</v>
+        <v>600</v>
       </c>
       <c r="F2335" t="n">
-        <v>1000000000</v>
+        <v>600000000</v>
       </c>
       <c r="G2335" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="H2335" t="n">
-        <v>1000000000</v>
+        <v>600000000</v>
       </c>
       <c r="I2335" t="n">
-        <v>1089400000</v>
+        <v>653640000</v>
       </c>
       <c r="J2335" t="n">
         <v>2023</v>
@@ -76939,7 +76939,7 @@
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>600 million euros</t>
+          <t>€1.65 million</t>
         </is>
       </c>
       <c r="B2336" t="inlineStr"/>
@@ -76952,33 +76952,33 @@
         </is>
       </c>
       <c r="E2336" t="n">
-        <v>600</v>
+        <v>1.65</v>
       </c>
       <c r="F2336" t="n">
-        <v>600000000</v>
+        <v>1650000</v>
       </c>
       <c r="G2336" s="2" t="n">
-        <v>44958</v>
+        <v>45323</v>
       </c>
       <c r="H2336" t="n">
-        <v>600000000</v>
+        <v>1650000</v>
       </c>
       <c r="I2336" t="n">
-        <v>653640000</v>
+        <v>1784310</v>
       </c>
       <c r="J2336" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>€1.65 million</t>
+          <t>€1.65 billion</t>
         </is>
       </c>
       <c r="B2337" t="inlineStr"/>
       <c r="C2337" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2337" t="inlineStr">
         <is>
@@ -76989,16 +76989,16 @@
         <v>1.65</v>
       </c>
       <c r="F2337" t="n">
-        <v>1650000</v>
+        <v>1650000000</v>
       </c>
       <c r="G2337" s="2" t="n">
-        <v>45323</v>
+        <v>45474</v>
       </c>
       <c r="H2337" t="n">
-        <v>1650000</v>
+        <v>1650000000</v>
       </c>
       <c r="I2337" t="n">
-        <v>1784310</v>
+        <v>1772925000</v>
       </c>
       <c r="J2337" t="n">
         <v>2024</v>
@@ -77041,7 +77041,7 @@
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>€1.65 billion</t>
+          <t>over £1 billion</t>
         </is>
       </c>
       <c r="B2339" t="inlineStr"/>
@@ -77050,32 +77050,40 @@
       </c>
       <c r="D2339" t="inlineStr">
         <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2339" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F2339" t="n">
-        <v>1650000000</v>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E2339" t="inlineStr">
+        <is>
+          <t>[1.0, None]</t>
+        </is>
+      </c>
+      <c r="F2339" t="inlineStr">
+        <is>
+          <t>[1000000000.0, None]</t>
+        </is>
       </c>
       <c r="G2339" s="2" t="n">
-        <v>45474</v>
-      </c>
-      <c r="H2339" t="n">
-        <v>1650000000</v>
-      </c>
-      <c r="I2339" t="n">
-        <v>1772925000</v>
+        <v>45108</v>
+      </c>
+      <c r="H2339" t="inlineStr">
+        <is>
+          <t>[1164433541.896319, None]</t>
+        </is>
+      </c>
+      <c r="I2339" t="inlineStr">
+        <is>
+          <t>[1266554363.5206263, None]</t>
+        </is>
       </c>
       <c r="J2339" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>over £1 billion</t>
+          <t>€1 billion</t>
         </is>
       </c>
       <c r="B2340" t="inlineStr"/>
@@ -77084,34 +77092,26 @@
       </c>
       <c r="D2340" t="inlineStr">
         <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="E2340" t="inlineStr">
-        <is>
-          <t>[1.0, None]</t>
-        </is>
-      </c>
-      <c r="F2340" t="inlineStr">
-        <is>
-          <t>[1000000000.0, None]</t>
-        </is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2340" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2340" t="n">
+        <v>1000000000</v>
       </c>
       <c r="G2340" s="2" t="n">
-        <v>45108</v>
-      </c>
-      <c r="H2340" t="inlineStr">
-        <is>
-          <t>[1164433541.896319, None]</t>
-        </is>
-      </c>
-      <c r="I2340" t="inlineStr">
-        <is>
-          <t>[1266554363.5206263, None]</t>
-        </is>
+        <v>44835</v>
+      </c>
+      <c r="H2340" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="I2340" t="n">
+        <v>975333333.3333334</v>
       </c>
       <c r="J2340" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2341">
@@ -77151,7 +77151,7 @@
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>€1 billion</t>
+          <t>€1.1 billion</t>
         </is>
       </c>
       <c r="B2342" t="inlineStr"/>
@@ -77164,22 +77164,22 @@
         </is>
       </c>
       <c r="E2342" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="F2342" t="n">
-        <v>1000000000</v>
+        <v>1100000000</v>
       </c>
       <c r="G2342" s="2" t="n">
-        <v>44835</v>
+        <v>44440</v>
       </c>
       <c r="H2342" t="n">
-        <v>1000000000</v>
+        <v>1100000000</v>
       </c>
       <c r="I2342" t="n">
-        <v>975333333.3333334</v>
+        <v>1299870000</v>
       </c>
       <c r="J2342" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="2343">
@@ -77219,12 +77219,12 @@
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>€1.1 billion</t>
+          <t>€ 13.6 million</t>
         </is>
       </c>
       <c r="B2344" t="inlineStr"/>
       <c r="C2344" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2344" t="inlineStr">
         <is>
@@ -77232,19 +77232,19 @@
         </is>
       </c>
       <c r="E2344" t="n">
-        <v>1.1</v>
+        <v>13.6</v>
       </c>
       <c r="F2344" t="n">
-        <v>1100000000</v>
+        <v>13600000</v>
       </c>
       <c r="G2344" s="2" t="n">
-        <v>44440</v>
+        <v>44317</v>
       </c>
       <c r="H2344" t="n">
-        <v>1100000000</v>
+        <v>13600000</v>
       </c>
       <c r="I2344" t="n">
-        <v>1299870000</v>
+        <v>16414293.33333333</v>
       </c>
       <c r="J2344" t="n">
         <v>2021</v>
@@ -77253,32 +77253,40 @@
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>€ 13.6 million</t>
+          <t>€1-1.5 billion</t>
         </is>
       </c>
       <c r="B2345" t="inlineStr"/>
       <c r="C2345" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2345" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="E2345" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="F2345" t="n">
-        <v>13600000</v>
+      <c r="E2345" t="inlineStr">
+        <is>
+          <t>[1.0, 1.5]</t>
+        </is>
+      </c>
+      <c r="F2345" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
       </c>
       <c r="G2345" s="2" t="n">
-        <v>44317</v>
-      </c>
-      <c r="H2345" t="n">
-        <v>13600000</v>
-      </c>
-      <c r="I2345" t="n">
-        <v>16414293.33333333</v>
+        <v>44256</v>
+      </c>
+      <c r="H2345" t="inlineStr">
+        <is>
+          <t>[1000000000.0, 1500000000.0]</t>
+        </is>
+      </c>
+      <c r="I2345" t="inlineStr">
+        <is>
+          <t>[1205300000.0, 1807950000.0]</t>
+        </is>
       </c>
       <c r="J2345" t="n">
         <v>2021</v>
@@ -77413,7 +77421,7 @@
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>€1-1.5 billion</t>
+          <t>SEK 3.1 billion</t>
         </is>
       </c>
       <c r="B2349" t="inlineStr"/>
@@ -77422,40 +77430,32 @@
       </c>
       <c r="D2349" t="inlineStr">
         <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2349" t="inlineStr">
-        <is>
-          <t>[1.0, 1.5]</t>
-        </is>
-      </c>
-      <c r="F2349" t="inlineStr">
-        <is>
-          <t>[1000000000.0, 1500000000.0]</t>
-        </is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E2349" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F2349" t="n">
+        <v>3100000000</v>
       </c>
       <c r="G2349" s="2" t="n">
-        <v>44256</v>
-      </c>
-      <c r="H2349" t="inlineStr">
-        <is>
-          <t>[1000000000.0, 1500000000.0]</t>
-        </is>
-      </c>
-      <c r="I2349" t="inlineStr">
-        <is>
-          <t>[1205300000.0, 1807950000.0]</t>
-        </is>
+        <v>45383</v>
+      </c>
+      <c r="H2349" t="n">
+        <v>268375032.4647217</v>
+      </c>
+      <c r="I2349" t="n">
+        <v>288809107.4365857</v>
       </c>
       <c r="J2349" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>SEK 3.1 billion</t>
+          <t>SEK 3,1 billion</t>
         </is>
       </c>
       <c r="B2350" t="inlineStr"/>
@@ -77474,22 +77474,22 @@
         <v>3100000000</v>
       </c>
       <c r="G2350" s="2" t="n">
-        <v>45383</v>
+        <v>45261</v>
       </c>
       <c r="H2350" t="n">
-        <v>268375032.4647217</v>
+        <v>272611352.943763</v>
       </c>
       <c r="I2350" t="n">
-        <v>288809107.4365857</v>
+        <v>296464846.3263422</v>
       </c>
       <c r="J2350" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>SEK 3,1 billion</t>
+          <t>SEK 3,7 billion</t>
         </is>
       </c>
       <c r="B2351" t="inlineStr"/>
@@ -77502,19 +77502,19 @@
         </is>
       </c>
       <c r="E2351" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
       <c r="F2351" t="n">
-        <v>3100000000</v>
+        <v>3700000000</v>
       </c>
       <c r="G2351" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="H2351" t="n">
-        <v>272611352.943763</v>
+        <v>325374840.6102977</v>
       </c>
       <c r="I2351" t="n">
-        <v>296464846.3263422</v>
+        <v>353845139.1636987</v>
       </c>
       <c r="J2351" t="n">
         <v>2023</v>
@@ -77523,7 +77523,7 @@
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>SEK 3,7 billion</t>
+          <t>SEK 6,2 billion</t>
         </is>
       </c>
       <c r="B2352" t="inlineStr"/>
@@ -77536,19 +77536,19 @@
         </is>
       </c>
       <c r="E2352" t="n">
-        <v>3.7</v>
+        <v>6.2</v>
       </c>
       <c r="F2352" t="n">
-        <v>3700000000</v>
+        <v>6200000000</v>
       </c>
       <c r="G2352" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="H2352" t="n">
-        <v>325374840.6102977</v>
+        <v>545222705.8875259</v>
       </c>
       <c r="I2352" t="n">
-        <v>353845139.1636987</v>
+        <v>592929692.6526843</v>
       </c>
       <c r="J2352" t="n">
         <v>2023</v>
@@ -77557,35 +77557,35 @@
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>SEK 6,2 billion</t>
+          <t>EUR 506 million</t>
         </is>
       </c>
       <c r="B2353" t="inlineStr"/>
       <c r="C2353" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2353" t="inlineStr">
         <is>
-          <t>SEK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="E2353" t="n">
-        <v>6.2</v>
+        <v>506</v>
       </c>
       <c r="F2353" t="n">
-        <v>6200000000</v>
+        <v>506000000</v>
       </c>
       <c r="G2353" s="2" t="n">
-        <v>45261</v>
+        <v>44621</v>
       </c>
       <c r="H2353" t="n">
-        <v>545222705.8875259</v>
+        <v>506000000</v>
       </c>
       <c r="I2353" t="n">
-        <v>592929692.6526843</v>
+        <v>564797200</v>
       </c>
       <c r="J2353" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2354">
@@ -77625,94 +77625,60 @@
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>EUR 506 million</t>
+          <t>CZK 1.4 billion (EUR 52 million)</t>
         </is>
       </c>
       <c r="B2355" t="inlineStr"/>
       <c r="C2355" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2355" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CZK</t>
         </is>
       </c>
       <c r="E2355" t="n">
-        <v>506</v>
+        <v>1.4</v>
       </c>
       <c r="F2355" t="n">
-        <v>506000000</v>
+        <v>1400000000</v>
       </c>
       <c r="G2355" s="2" t="n">
-        <v>44621</v>
+        <v>44075</v>
       </c>
       <c r="H2355" t="n">
-        <v>506000000</v>
+        <v>53382139.86120643</v>
       </c>
       <c r="I2355" t="n">
-        <v>564797200</v>
+        <v>63989171.05162816</v>
       </c>
       <c r="J2355" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>CZK 1.4 billion (EUR 52 million)</t>
+          <t>30 billion-krona ($2.8 billion)</t>
         </is>
       </c>
       <c r="B2356" t="inlineStr"/>
       <c r="C2356" t="n">
         <v>1000000000</v>
       </c>
-      <c r="D2356" t="inlineStr">
-        <is>
-          <t>CZK</t>
-        </is>
-      </c>
+      <c r="D2356" t="inlineStr"/>
       <c r="E2356" t="n">
-        <v>1.4</v>
+        <v>30</v>
       </c>
       <c r="F2356" t="n">
-        <v>1400000000</v>
+        <v>30000000000</v>
       </c>
       <c r="G2356" s="2" t="n">
-        <v>44075</v>
-      </c>
-      <c r="H2356" t="n">
-        <v>53382139.86120643</v>
-      </c>
-      <c r="I2356" t="n">
-        <v>63989171.05162816</v>
-      </c>
+        <v>45658</v>
+      </c>
+      <c r="H2356" t="inlineStr"/>
+      <c r="I2356" t="inlineStr"/>
       <c r="J2356" t="n">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="2357">
-      <c r="A2357" t="inlineStr">
-        <is>
-          <t>30 billion-krona ($2.8 billion)</t>
-        </is>
-      </c>
-      <c r="B2357" t="inlineStr"/>
-      <c r="C2357" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="D2357" t="inlineStr"/>
-      <c r="E2357" t="n">
-        <v>30</v>
-      </c>
-      <c r="F2357" t="n">
-        <v>30000000000</v>
-      </c>
-      <c r="G2357" s="2" t="n">
-        <v>45658</v>
-      </c>
-      <c r="H2357" t="inlineStr"/>
-      <c r="I2357" t="inlineStr"/>
-      <c r="J2357" t="n">
         <v>2025</v>
       </c>
     </row>

</xml_diff>

<commit_message>
main is updated from phase summaries
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/check_investments.xlsx
+++ b/reconcile/storage/output/check_investments.xlsx
@@ -59915,34 +59915,32 @@
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
-          <t>US$1.1bn</t>
-        </is>
-      </c>
-      <c r="B1832" t="inlineStr">
-        <is>
-          <t>1bn</t>
-        </is>
-      </c>
-      <c r="C1832" t="inlineStr"/>
+          <t>$1.1 billion</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr"/>
+      <c r="C1832" t="n">
+        <v>1000000000</v>
+      </c>
       <c r="D1832" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
       <c r="E1832" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="F1832" t="n">
-        <v>1</v>
+        <v>1100000000</v>
       </c>
       <c r="G1832" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="H1832" t="n">
-        <v>0.9306654257794322</v>
+        <v>1023731968.357376</v>
       </c>
       <c r="I1832" t="n">
-        <v>1</v>
+        <v>1100000000</v>
       </c>
       <c r="J1832" t="n">
         <v>2024</v>

</xml_diff>

<commit_message>
cleaning product_lv2 iron in group.py
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/check_investments.xlsx
+++ b/reconcile/storage/output/check_investments.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2427"/>
+  <dimension ref="A1:J2426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78445,127 +78445,127 @@
       </c>
     </row>
     <row r="2379">
-      <c r="A2379" t="inlineStr">
-        <is>
-          <t>HUF 15 bln</t>
-        </is>
-      </c>
+      <c r="A2379" t="inlineStr"/>
       <c r="B2379" t="inlineStr"/>
-      <c r="C2379" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="D2379" t="inlineStr">
-        <is>
-          <t>HUF</t>
-        </is>
-      </c>
-      <c r="E2379" t="n">
-        <v>15</v>
-      </c>
-      <c r="F2379" t="n">
-        <v>15000000000</v>
-      </c>
+      <c r="C2379" t="inlineStr"/>
+      <c r="D2379" t="inlineStr"/>
+      <c r="E2379" t="inlineStr"/>
+      <c r="F2379" t="inlineStr"/>
       <c r="G2379" s="2" t="n">
-        <v>41883</v>
-      </c>
-      <c r="H2379" t="n">
-        <v>47732697</v>
-      </c>
-      <c r="I2379" t="n">
-        <v>62687351</v>
-      </c>
+        <v>41306</v>
+      </c>
+      <c r="H2379" t="inlineStr"/>
+      <c r="I2379" t="inlineStr"/>
       <c r="J2379" t="n">
-        <v>2014</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="2380">
-      <c r="A2380" t="inlineStr"/>
+      <c r="A2380" t="inlineStr">
+        <is>
+          <t>€53 million ($57.4 million)</t>
+        </is>
+      </c>
       <c r="B2380" t="inlineStr"/>
-      <c r="C2380" t="inlineStr"/>
-      <c r="D2380" t="inlineStr"/>
-      <c r="E2380" t="inlineStr"/>
-      <c r="F2380" t="inlineStr"/>
+      <c r="C2380" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2380" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2380" t="n">
+        <v>53</v>
+      </c>
+      <c r="F2380" t="n">
+        <v>53000000</v>
+      </c>
       <c r="G2380" s="2" t="n">
-        <v>41306</v>
-      </c>
-      <c r="H2380" t="inlineStr"/>
-      <c r="I2380" t="inlineStr"/>
+        <v>45566</v>
+      </c>
+      <c r="H2380" t="n">
+        <v>53000000</v>
+      </c>
+      <c r="I2380" t="n">
+        <v>58755800</v>
+      </c>
       <c r="J2380" t="n">
-        <v>2013</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>€53 million ($57.4 million)</t>
+          <t>PLN 1 billion</t>
         </is>
       </c>
       <c r="B2381" t="inlineStr"/>
       <c r="C2381" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2381" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>PLN</t>
         </is>
       </c>
       <c r="E2381" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F2381" t="n">
-        <v>53000000</v>
+        <v>1000000000</v>
       </c>
       <c r="G2381" s="2" t="n">
-        <v>45566</v>
+        <v>44197</v>
       </c>
       <c r="H2381" t="n">
-        <v>53000000</v>
+        <v>219459471</v>
       </c>
       <c r="I2381" t="n">
-        <v>58755800</v>
+        <v>269435879</v>
       </c>
       <c r="J2381" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>PLN 1 billion</t>
+          <t>€90 million</t>
         </is>
       </c>
       <c r="B2382" t="inlineStr"/>
       <c r="C2382" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2382" t="inlineStr">
         <is>
-          <t>PLN</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="E2382" t="n">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="F2382" t="n">
-        <v>1000000000</v>
+        <v>90000000</v>
       </c>
       <c r="G2382" s="2" t="n">
-        <v>44197</v>
+        <v>44986</v>
       </c>
       <c r="H2382" t="n">
-        <v>219459471</v>
+        <v>90000000</v>
       </c>
       <c r="I2382" t="n">
-        <v>269435879</v>
+        <v>96156000</v>
       </c>
       <c r="J2382" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>€90 million</t>
+          <t>€21 million</t>
         </is>
       </c>
       <c r="B2383" t="inlineStr"/>
@@ -78578,28 +78578,28 @@
         </is>
       </c>
       <c r="E2383" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="F2383" t="n">
-        <v>90000000</v>
+        <v>21000000</v>
       </c>
       <c r="G2383" s="2" t="n">
-        <v>44986</v>
+        <v>44440</v>
       </c>
       <c r="H2383" t="n">
-        <v>90000000</v>
+        <v>21000000</v>
       </c>
       <c r="I2383" t="n">
-        <v>96156000</v>
+        <v>24815700</v>
       </c>
       <c r="J2383" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>€21 million</t>
+          <t>€10 million ($11.3 million)</t>
         </is>
       </c>
       <c r="B2384" t="inlineStr"/>
@@ -78612,28 +78612,28 @@
         </is>
       </c>
       <c r="E2384" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F2384" t="n">
-        <v>21000000</v>
+        <v>10000000</v>
       </c>
       <c r="G2384" s="2" t="n">
-        <v>44440</v>
+        <v>46874</v>
       </c>
       <c r="H2384" t="n">
-        <v>21000000</v>
+        <v>10000000</v>
       </c>
       <c r="I2384" t="n">
-        <v>24815700</v>
+        <v>11654000</v>
       </c>
       <c r="J2384" t="n">
-        <v>2021</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>€10 million ($11.3 million)</t>
+          <t>20 million euros</t>
         </is>
       </c>
       <c r="B2385" t="inlineStr"/>
@@ -78646,22 +78646,22 @@
         </is>
       </c>
       <c r="E2385" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F2385" t="n">
-        <v>10000000</v>
+        <v>20000000</v>
       </c>
       <c r="G2385" s="2" t="n">
-        <v>46874</v>
+        <v>45200</v>
       </c>
       <c r="H2385" t="n">
-        <v>10000000</v>
+        <v>20000000</v>
       </c>
       <c r="I2385" t="n">
-        <v>11654000</v>
+        <v>21102667</v>
       </c>
       <c r="J2385" t="n">
-        <v>2028</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2386">
@@ -78769,7 +78769,7 @@
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>20 million euros</t>
+          <t>€1.2M</t>
         </is>
       </c>
       <c r="B2389" t="inlineStr"/>
@@ -78782,28 +78782,28 @@
         </is>
       </c>
       <c r="E2389" t="n">
-        <v>20</v>
+        <v>1.2</v>
       </c>
       <c r="F2389" t="n">
-        <v>20000000</v>
+        <v>1200000</v>
       </c>
       <c r="G2389" s="2" t="n">
-        <v>45200</v>
+        <v>45323</v>
       </c>
       <c r="H2389" t="n">
-        <v>20000000</v>
+        <v>1200000</v>
       </c>
       <c r="I2389" t="n">
-        <v>21102667</v>
+        <v>1297680</v>
       </c>
       <c r="J2389" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>€1.2M</t>
+          <t>€10 million</t>
         </is>
       </c>
       <c r="B2390" t="inlineStr"/>
@@ -78816,28 +78816,28 @@
         </is>
       </c>
       <c r="E2390" t="n">
-        <v>1.2</v>
+        <v>10</v>
       </c>
       <c r="F2390" t="n">
-        <v>1200000</v>
+        <v>10000000</v>
       </c>
       <c r="G2390" s="2" t="n">
-        <v>45323</v>
+        <v>45748</v>
       </c>
       <c r="H2390" t="n">
-        <v>1200000</v>
+        <v>10000000</v>
       </c>
       <c r="I2390" t="n">
-        <v>1297680</v>
+        <v>10788000</v>
       </c>
       <c r="J2390" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>€10 million</t>
+          <t>€4.2 million ($4.6 million)</t>
         </is>
       </c>
       <c r="B2391" t="inlineStr"/>
@@ -78850,19 +78850,19 @@
         </is>
       </c>
       <c r="E2391" t="n">
-        <v>10</v>
+        <v>4.2</v>
       </c>
       <c r="F2391" t="n">
-        <v>10000000</v>
+        <v>4200000</v>
       </c>
       <c r="G2391" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="H2391" t="n">
-        <v>10000000</v>
+        <v>4200000</v>
       </c>
       <c r="I2391" t="n">
-        <v>10788000</v>
+        <v>4530960</v>
       </c>
       <c r="J2391" t="n">
         <v>2025</v>
@@ -78871,7 +78871,7 @@
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>€4.2 million ($4.6 million)</t>
+          <t>€4.2 million</t>
         </is>
       </c>
       <c r="B2392" t="inlineStr"/>
@@ -78890,72 +78890,72 @@
         <v>4200000</v>
       </c>
       <c r="G2392" s="2" t="n">
-        <v>45748</v>
+        <v>45566</v>
       </c>
       <c r="H2392" t="n">
         <v>4200000</v>
       </c>
       <c r="I2392" t="n">
-        <v>4530960</v>
+        <v>4656120</v>
       </c>
       <c r="J2392" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" t="inlineStr"/>
+      <c r="B2393" t="inlineStr"/>
+      <c r="C2393" t="inlineStr"/>
+      <c r="D2393" t="inlineStr"/>
+      <c r="E2393" t="inlineStr"/>
+      <c r="F2393" t="inlineStr"/>
+      <c r="G2393" s="2" t="n">
+        <v>44682</v>
+      </c>
+      <c r="H2393" t="inlineStr"/>
+      <c r="I2393" t="inlineStr"/>
+      <c r="J2393" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" t="inlineStr">
+        <is>
+          <t>€60 million</t>
+        </is>
+      </c>
+      <c r="B2394" t="inlineStr"/>
+      <c r="C2394" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2394" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2394" t="n">
+        <v>60</v>
+      </c>
+      <c r="F2394" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="G2394" s="2" t="n">
+        <v>45931</v>
+      </c>
+      <c r="H2394" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="I2394" t="n">
+        <v>69924000</v>
+      </c>
+      <c r="J2394" t="n">
         <v>2025</v>
-      </c>
-    </row>
-    <row r="2393">
-      <c r="A2393" t="inlineStr">
-        <is>
-          <t>€4.2 million</t>
-        </is>
-      </c>
-      <c r="B2393" t="inlineStr"/>
-      <c r="C2393" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D2393" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2393" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F2393" t="n">
-        <v>4200000</v>
-      </c>
-      <c r="G2393" s="2" t="n">
-        <v>45566</v>
-      </c>
-      <c r="H2393" t="n">
-        <v>4200000</v>
-      </c>
-      <c r="I2393" t="n">
-        <v>4656120</v>
-      </c>
-      <c r="J2393" t="n">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="2394">
-      <c r="A2394" t="inlineStr"/>
-      <c r="B2394" t="inlineStr"/>
-      <c r="C2394" t="inlineStr"/>
-      <c r="D2394" t="inlineStr"/>
-      <c r="E2394" t="inlineStr"/>
-      <c r="F2394" t="inlineStr"/>
-      <c r="G2394" s="2" t="n">
-        <v>44682</v>
-      </c>
-      <c r="H2394" t="inlineStr"/>
-      <c r="I2394" t="inlineStr"/>
-      <c r="J2394" t="n">
-        <v>2022</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>€60 million</t>
+          <t>€85.6 million</t>
         </is>
       </c>
       <c r="B2395" t="inlineStr"/>
@@ -78968,22 +78968,22 @@
         </is>
       </c>
       <c r="E2395" t="n">
-        <v>60</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="F2395" t="n">
-        <v>60000000</v>
+        <v>85600000</v>
       </c>
       <c r="G2395" s="2" t="n">
-        <v>45931</v>
+        <v>43525</v>
       </c>
       <c r="H2395" t="n">
-        <v>60000000</v>
+        <v>85600000</v>
       </c>
       <c r="I2395" t="n">
-        <v>69924000</v>
+        <v>97438480</v>
       </c>
       <c r="J2395" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="2396">
@@ -79023,7 +79023,7 @@
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>€85.6 million</t>
+          <t>€20 million</t>
         </is>
       </c>
       <c r="B2397" t="inlineStr"/>
@@ -79036,28 +79036,28 @@
         </is>
       </c>
       <c r="E2397" t="n">
-        <v>85.59999999999999</v>
+        <v>20</v>
       </c>
       <c r="F2397" t="n">
-        <v>85600000</v>
+        <v>20000000</v>
       </c>
       <c r="G2397" s="2" t="n">
-        <v>43525</v>
+        <v>44105</v>
       </c>
       <c r="H2397" t="n">
-        <v>85600000</v>
+        <v>20000000</v>
       </c>
       <c r="I2397" t="n">
-        <v>97438480</v>
+        <v>23504000</v>
       </c>
       <c r="J2397" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>€20 million</t>
+          <t>€170m</t>
         </is>
       </c>
       <c r="B2398" t="inlineStr"/>
@@ -79070,22 +79070,22 @@
         </is>
       </c>
       <c r="E2398" t="n">
-        <v>20</v>
+        <v>170</v>
       </c>
       <c r="F2398" t="n">
-        <v>20000000</v>
+        <v>170000000</v>
       </c>
       <c r="G2398" s="2" t="n">
-        <v>44105</v>
+        <v>45778</v>
       </c>
       <c r="H2398" t="n">
-        <v>20000000</v>
+        <v>170000000</v>
       </c>
       <c r="I2398" t="n">
-        <v>23504000</v>
+        <v>193086000</v>
       </c>
       <c r="J2398" t="n">
-        <v>2020</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="2399">
@@ -79125,7 +79125,7 @@
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>€170m</t>
+          <t>€50m</t>
         </is>
       </c>
       <c r="B2400" t="inlineStr"/>
@@ -79138,19 +79138,19 @@
         </is>
       </c>
       <c r="E2400" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="F2400" t="n">
-        <v>170000000</v>
+        <v>50000000</v>
       </c>
       <c r="G2400" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="H2400" t="n">
-        <v>170000000</v>
+        <v>50000000</v>
       </c>
       <c r="I2400" t="n">
-        <v>193086000</v>
+        <v>56790000</v>
       </c>
       <c r="J2400" t="n">
         <v>2025</v>
@@ -79159,7 +79159,7 @@
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>€50m</t>
+          <t>€32.3 million</t>
         </is>
       </c>
       <c r="B2401" t="inlineStr"/>
@@ -79172,28 +79172,28 @@
         </is>
       </c>
       <c r="E2401" t="n">
-        <v>50</v>
+        <v>32.3</v>
       </c>
       <c r="F2401" t="n">
-        <v>50000000</v>
+        <v>32300000</v>
       </c>
       <c r="G2401" s="2" t="n">
-        <v>45778</v>
+        <v>45383</v>
       </c>
       <c r="H2401" t="n">
-        <v>50000000</v>
+        <v>32300000</v>
       </c>
       <c r="I2401" t="n">
-        <v>56790000</v>
+        <v>34759322</v>
       </c>
       <c r="J2401" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>€32.3 million</t>
+          <t>EUR 22m</t>
         </is>
       </c>
       <c r="B2402" t="inlineStr"/>
@@ -79206,22 +79206,22 @@
         </is>
       </c>
       <c r="E2402" t="n">
-        <v>32.3</v>
+        <v>22</v>
       </c>
       <c r="F2402" t="n">
-        <v>32300000</v>
+        <v>22000000</v>
       </c>
       <c r="G2402" s="2" t="n">
-        <v>45383</v>
+        <v>45809</v>
       </c>
       <c r="H2402" t="n">
-        <v>32300000</v>
+        <v>22000000</v>
       </c>
       <c r="I2402" t="n">
-        <v>34759322</v>
+        <v>25063133</v>
       </c>
       <c r="J2402" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="2403">
@@ -79295,7 +79295,7 @@
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>EUR 22m</t>
+          <t>30 million euros ($33 million)</t>
         </is>
       </c>
       <c r="B2405" t="inlineStr"/>
@@ -79308,28 +79308,28 @@
         </is>
       </c>
       <c r="E2405" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F2405" t="n">
-        <v>22000000</v>
+        <v>30000000</v>
       </c>
       <c r="G2405" s="2" t="n">
-        <v>45809</v>
+        <v>45047</v>
       </c>
       <c r="H2405" t="n">
-        <v>22000000</v>
+        <v>30000000</v>
       </c>
       <c r="I2405" t="n">
-        <v>25063133</v>
+        <v>32907000</v>
       </c>
       <c r="J2405" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>30 million euros ($33 million)</t>
+          <t>€30M</t>
         </is>
       </c>
       <c r="B2406" t="inlineStr"/>
@@ -79361,53 +79361,53 @@
       </c>
     </row>
     <row r="2407">
-      <c r="A2407" t="inlineStr">
-        <is>
-          <t>€30M</t>
-        </is>
-      </c>
+      <c r="A2407" t="inlineStr"/>
       <c r="B2407" t="inlineStr"/>
-      <c r="C2407" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D2407" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2407" t="n">
-        <v>30</v>
-      </c>
-      <c r="F2407" t="n">
-        <v>30000000</v>
-      </c>
+      <c r="C2407" t="inlineStr"/>
+      <c r="D2407" t="inlineStr"/>
+      <c r="E2407" t="inlineStr"/>
+      <c r="F2407" t="inlineStr"/>
       <c r="G2407" s="2" t="n">
-        <v>45047</v>
-      </c>
-      <c r="H2407" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="I2407" t="n">
-        <v>32907000</v>
-      </c>
+        <v>44805</v>
+      </c>
+      <c r="H2407" t="inlineStr"/>
+      <c r="I2407" t="inlineStr"/>
       <c r="J2407" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2408">
-      <c r="A2408" t="inlineStr"/>
+      <c r="A2408" t="inlineStr">
+        <is>
+          <t>SEK 1.2 billion</t>
+        </is>
+      </c>
       <c r="B2408" t="inlineStr"/>
-      <c r="C2408" t="inlineStr"/>
-      <c r="D2408" t="inlineStr"/>
-      <c r="E2408" t="inlineStr"/>
-      <c r="F2408" t="inlineStr"/>
+      <c r="C2408" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2408" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E2408" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F2408" t="n">
+        <v>1200000000</v>
+      </c>
       <c r="G2408" s="2" t="n">
-        <v>44805</v>
-      </c>
-      <c r="H2408" t="inlineStr"/>
-      <c r="I2408" t="inlineStr"/>
+        <v>45536</v>
+      </c>
+      <c r="H2408" t="n">
+        <v>105765700</v>
+      </c>
+      <c r="I2408" t="n">
+        <v>117079104</v>
+      </c>
       <c r="J2408" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="2409">
@@ -79447,41 +79447,41 @@
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>SEK 1.2 billion</t>
+          <t>160 million euros</t>
         </is>
       </c>
       <c r="B2410" t="inlineStr"/>
       <c r="C2410" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2410" t="inlineStr">
         <is>
-          <t>SEK</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="E2410" t="n">
-        <v>1.2</v>
+        <v>160</v>
       </c>
       <c r="F2410" t="n">
-        <v>1200000000</v>
+        <v>160000000</v>
       </c>
       <c r="G2410" s="2" t="n">
-        <v>45536</v>
+        <v>45078</v>
       </c>
       <c r="H2410" t="n">
-        <v>105765700</v>
+        <v>160000000</v>
       </c>
       <c r="I2410" t="n">
-        <v>117079104</v>
+        <v>171152000</v>
       </c>
       <c r="J2410" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>160 million euros</t>
+          <t>€160 million ($176 million)</t>
         </is>
       </c>
       <c r="B2411" t="inlineStr"/>
@@ -79617,7 +79617,7 @@
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>€160 million ($176 million)</t>
+          <t>€150 million</t>
         </is>
       </c>
       <c r="B2415" t="inlineStr"/>
@@ -79630,28 +79630,28 @@
         </is>
       </c>
       <c r="E2415" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F2415" t="n">
-        <v>160000000</v>
+        <v>150000000</v>
       </c>
       <c r="G2415" s="2" t="n">
-        <v>45078</v>
+        <v>43313</v>
       </c>
       <c r="H2415" t="n">
-        <v>160000000</v>
+        <v>150000000</v>
       </c>
       <c r="I2415" t="n">
-        <v>171152000</v>
+        <v>175440000</v>
       </c>
       <c r="J2415" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>€150 million</t>
+          <t>200 million euros</t>
         </is>
       </c>
       <c r="B2416" t="inlineStr"/>
@@ -79664,22 +79664,22 @@
         </is>
       </c>
       <c r="E2416" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F2416" t="n">
-        <v>150000000</v>
+        <v>200000000</v>
       </c>
       <c r="G2416" s="2" t="n">
-        <v>43313</v>
+        <v>44805</v>
       </c>
       <c r="H2416" t="n">
-        <v>150000000</v>
+        <v>200000000</v>
       </c>
       <c r="I2416" t="n">
-        <v>175440000</v>
+        <v>200080000</v>
       </c>
       <c r="J2416" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2417">
@@ -79701,16 +79701,16 @@
         <v>200</v>
       </c>
       <c r="F2417" t="n">
-        <v>200000000</v>
+        <v>100000000</v>
       </c>
       <c r="G2417" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="H2417" t="n">
-        <v>200000000</v>
+        <v>100000000</v>
       </c>
       <c r="I2417" t="n">
-        <v>200080000</v>
+        <v>100040000</v>
       </c>
       <c r="J2417" t="n">
         <v>2022</v>
@@ -79787,7 +79787,7 @@
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>200 million euros</t>
+          <t>33 million euros</t>
         </is>
       </c>
       <c r="B2420" t="inlineStr"/>
@@ -79800,19 +79800,19 @@
         </is>
       </c>
       <c r="E2420" t="n">
-        <v>200</v>
+        <v>33</v>
       </c>
       <c r="F2420" t="n">
-        <v>100000000</v>
+        <v>33000000</v>
       </c>
       <c r="G2420" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="H2420" t="n">
-        <v>100000000</v>
+        <v>33000000</v>
       </c>
       <c r="I2420" t="n">
-        <v>100040000</v>
+        <v>33013200</v>
       </c>
       <c r="J2420" t="n">
         <v>2022</v>
@@ -79821,7 +79821,7 @@
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>33 million euros</t>
+          <t>€35 million</t>
         </is>
       </c>
       <c r="B2421" t="inlineStr"/>
@@ -79834,22 +79834,22 @@
         </is>
       </c>
       <c r="E2421" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F2421" t="n">
-        <v>33000000</v>
+        <v>35000000</v>
       </c>
       <c r="G2421" s="2" t="n">
-        <v>44805</v>
+        <v>45901</v>
       </c>
       <c r="H2421" t="n">
-        <v>33000000</v>
+        <v>35000000</v>
       </c>
       <c r="I2421" t="n">
-        <v>33013200</v>
+        <v>40789000</v>
       </c>
       <c r="J2421" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="2422">
@@ -79889,7 +79889,7 @@
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>€35 million</t>
+          <t>up to USD $320 million</t>
         </is>
       </c>
       <c r="B2423" t="inlineStr"/>
@@ -79898,23 +79898,31 @@
       </c>
       <c r="D2423" t="inlineStr">
         <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2423" t="n">
-        <v>35</v>
-      </c>
-      <c r="F2423" t="n">
-        <v>35000000</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E2423" t="inlineStr">
+        <is>
+          <t>[None, 320.0]</t>
+        </is>
+      </c>
+      <c r="F2423" t="inlineStr">
+        <is>
+          <t>[None, 320000000.0]</t>
+        </is>
       </c>
       <c r="G2423" s="2" t="n">
-        <v>45901</v>
-      </c>
-      <c r="H2423" t="n">
-        <v>35000000</v>
-      </c>
-      <c r="I2423" t="n">
-        <v>40789000</v>
+        <v>45778</v>
+      </c>
+      <c r="H2423" t="inlineStr">
+        <is>
+          <t>[None, 281739743.0]</t>
+        </is>
+      </c>
+      <c r="I2423" t="inlineStr">
+        <is>
+          <t>[None, 320000000.0]</t>
+        </is>
       </c>
       <c r="J2423" t="n">
         <v>2025</v>
@@ -79923,40 +79931,32 @@
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>up to USD $320 million</t>
+          <t>€2 billion</t>
         </is>
       </c>
       <c r="B2424" t="inlineStr"/>
       <c r="C2424" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
       <c r="D2424" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E2424" t="inlineStr">
-        <is>
-          <t>[None, 320.0]</t>
-        </is>
-      </c>
-      <c r="F2424" t="inlineStr">
-        <is>
-          <t>[None, 320000000.0]</t>
-        </is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2424" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2424" t="n">
+        <v>2000000000</v>
       </c>
       <c r="G2424" s="2" t="n">
-        <v>45778</v>
-      </c>
-      <c r="H2424" t="inlineStr">
-        <is>
-          <t>[None, 281739743.0]</t>
-        </is>
-      </c>
-      <c r="I2424" t="inlineStr">
-        <is>
-          <t>[None, 320000000.0]</t>
-        </is>
+        <v>45689</v>
+      </c>
+      <c r="H2424" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="I2424" t="n">
+        <v>2070666667</v>
       </c>
       <c r="J2424" t="n">
         <v>2025</v>
@@ -79999,12 +79999,12 @@
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>€2 billion</t>
+          <t>EUR 150 million</t>
         </is>
       </c>
       <c r="B2426" t="inlineStr"/>
       <c r="C2426" t="n">
-        <v>1000000000</v>
+        <v>1000000</v>
       </c>
       <c r="D2426" t="inlineStr">
         <is>
@@ -80012,55 +80012,21 @@
         </is>
       </c>
       <c r="E2426" t="n">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="F2426" t="n">
-        <v>2000000000</v>
+        <v>150000000</v>
       </c>
       <c r="G2426" s="2" t="n">
-        <v>45689</v>
+        <v>44531</v>
       </c>
       <c r="H2426" t="n">
-        <v>2000000000</v>
+        <v>150000000</v>
       </c>
       <c r="I2426" t="n">
-        <v>2070666667</v>
+        <v>169710000</v>
       </c>
       <c r="J2426" t="n">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="2427">
-      <c r="A2427" t="inlineStr">
-        <is>
-          <t>EUR 150 million</t>
-        </is>
-      </c>
-      <c r="B2427" t="inlineStr"/>
-      <c r="C2427" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D2427" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E2427" t="n">
-        <v>150</v>
-      </c>
-      <c r="F2427" t="n">
-        <v>150000000</v>
-      </c>
-      <c r="G2427" s="2" t="n">
-        <v>44531</v>
-      </c>
-      <c r="H2427" t="n">
-        <v>150000000</v>
-      </c>
-      <c r="I2427" t="n">
-        <v>169710000</v>
-      </c>
-      <c r="J2427" t="n">
         <v>2021</v>
       </c>
     </row>

</xml_diff>